<commit_message>
Update workout data and more compact UI changes
</commit_message>
<xml_diff>
--- a/data_samples/workout_entry_template.xlsx
+++ b/data_samples/workout_entry_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amlim/Downloads/azure-fit-platform/data_samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98978BD8-9387-614B-B63C-35F326FA0BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D815A4A9-A855-DE47-93E8-342CC5197530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{5828482D-6AAB-A34A-A077-81D95F329610}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16140" xr2:uid="{5828482D-6AAB-A34A-A077-81D95F329610}"/>
   </bookViews>
   <sheets>
     <sheet name="workout_entry_template" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1962" uniqueCount="217">
   <si>
     <t>date</t>
   </si>
@@ -658,6 +658,21 @@
   </si>
   <si>
     <t>Band-Assisted Tuck Planche</t>
+  </si>
+  <si>
+    <t>Calf Press</t>
+  </si>
+  <si>
+    <t>Curtsy Lunges</t>
+  </si>
+  <si>
+    <t>Lower Back Extensions</t>
+  </si>
+  <si>
+    <t>Standing Calf Raises</t>
+  </si>
+  <si>
+    <t>Baseball Swings</t>
   </si>
 </sst>
 </file>
@@ -1528,7 +1543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09805D65-2793-1C46-AB3E-4E9435A12762}">
-  <dimension ref="A1:H573"/>
+  <dimension ref="A1:H635"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -14729,6 +14744,1432 @@
       </c>
       <c r="G573" t="s">
         <v>125</v>
+      </c>
+    </row>
+    <row r="574" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A574" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B574" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C574" t="s">
+        <v>105</v>
+      </c>
+      <c r="D574">
+        <v>1</v>
+      </c>
+      <c r="E574">
+        <v>10</v>
+      </c>
+      <c r="F574">
+        <v>0</v>
+      </c>
+      <c r="G574" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="575" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A575" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B575" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C575" t="s">
+        <v>105</v>
+      </c>
+      <c r="D575">
+        <v>1</v>
+      </c>
+      <c r="E575">
+        <v>12</v>
+      </c>
+      <c r="F575">
+        <v>0</v>
+      </c>
+      <c r="G575" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="576" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A576" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B576" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C576" t="s">
+        <v>105</v>
+      </c>
+      <c r="D576">
+        <v>1</v>
+      </c>
+      <c r="E576">
+        <v>12</v>
+      </c>
+      <c r="F576">
+        <v>0</v>
+      </c>
+      <c r="G576" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="577" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A577" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B577" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C577" t="s">
+        <v>105</v>
+      </c>
+      <c r="D577">
+        <v>1</v>
+      </c>
+      <c r="E577">
+        <v>12</v>
+      </c>
+      <c r="F577">
+        <v>0</v>
+      </c>
+      <c r="G577" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="578" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A578" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B578" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C578" t="s">
+        <v>103</v>
+      </c>
+      <c r="D578">
+        <v>3</v>
+      </c>
+      <c r="E578">
+        <v>8</v>
+      </c>
+      <c r="F578">
+        <v>264</v>
+      </c>
+      <c r="G578" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="579" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A579" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B579" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C579" t="s">
+        <v>103</v>
+      </c>
+      <c r="D579">
+        <v>2</v>
+      </c>
+      <c r="E579">
+        <v>10</v>
+      </c>
+      <c r="F579">
+        <v>120</v>
+      </c>
+      <c r="G579" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="580" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A580" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B580" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C580" t="s">
+        <v>103</v>
+      </c>
+      <c r="D580">
+        <v>2</v>
+      </c>
+      <c r="E580">
+        <v>8</v>
+      </c>
+      <c r="F580">
+        <v>140</v>
+      </c>
+      <c r="G580" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="581" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A581" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B581" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C581" t="s">
+        <v>103</v>
+      </c>
+      <c r="D581">
+        <v>3</v>
+      </c>
+      <c r="E581">
+        <v>10</v>
+      </c>
+      <c r="F581">
+        <v>120</v>
+      </c>
+      <c r="G581" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="582" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A582" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B582" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C582" t="s">
+        <v>103</v>
+      </c>
+      <c r="D582">
+        <v>4</v>
+      </c>
+      <c r="E582">
+        <v>12</v>
+      </c>
+      <c r="F582">
+        <v>205</v>
+      </c>
+      <c r="G582" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="583" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A583" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B583" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C583" t="s">
+        <v>103</v>
+      </c>
+      <c r="D583">
+        <v>2</v>
+      </c>
+      <c r="E583">
+        <v>10</v>
+      </c>
+      <c r="F583">
+        <v>100</v>
+      </c>
+      <c r="G583" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="584" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A584" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B584" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C584" t="s">
+        <v>103</v>
+      </c>
+      <c r="D584">
+        <v>2</v>
+      </c>
+      <c r="E584">
+        <v>6</v>
+      </c>
+      <c r="F584">
+        <v>110</v>
+      </c>
+      <c r="G584" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="585" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A585" s="1">
+        <v>46041</v>
+      </c>
+      <c r="B585" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C585" t="s">
+        <v>103</v>
+      </c>
+      <c r="D585">
+        <v>4</v>
+      </c>
+      <c r="E585">
+        <v>12</v>
+      </c>
+      <c r="F585">
+        <v>130</v>
+      </c>
+      <c r="G585" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="586" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A586" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B586" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C586" t="s">
+        <v>105</v>
+      </c>
+      <c r="D586">
+        <v>2</v>
+      </c>
+      <c r="E586">
+        <v>15</v>
+      </c>
+      <c r="F586">
+        <v>0</v>
+      </c>
+      <c r="G586" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="587" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A587" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B587" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C587" t="s">
+        <v>105</v>
+      </c>
+      <c r="D587">
+        <v>2</v>
+      </c>
+      <c r="E587">
+        <v>15</v>
+      </c>
+      <c r="F587">
+        <v>0</v>
+      </c>
+      <c r="G587" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="588" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A588" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B588" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C588" t="s">
+        <v>104</v>
+      </c>
+      <c r="D588">
+        <v>3</v>
+      </c>
+      <c r="E588">
+        <v>15</v>
+      </c>
+      <c r="F588">
+        <v>0</v>
+      </c>
+      <c r="G588" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="589" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A589" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B589" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C589" t="s">
+        <v>103</v>
+      </c>
+      <c r="D589">
+        <v>3</v>
+      </c>
+      <c r="E589">
+        <v>15</v>
+      </c>
+      <c r="F589">
+        <v>0</v>
+      </c>
+      <c r="G589" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="590" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A590" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B590" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C590" t="s">
+        <v>98</v>
+      </c>
+      <c r="D590">
+        <v>4</v>
+      </c>
+      <c r="E590">
+        <v>30</v>
+      </c>
+      <c r="F590">
+        <v>0</v>
+      </c>
+      <c r="G590" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="591" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A591" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B591" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C591" t="s">
+        <v>98</v>
+      </c>
+      <c r="D591">
+        <v>3</v>
+      </c>
+      <c r="E591">
+        <v>6</v>
+      </c>
+      <c r="F591">
+        <v>0</v>
+      </c>
+      <c r="G591" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="592" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A592" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B592" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C592" t="s">
+        <v>103</v>
+      </c>
+      <c r="D592">
+        <v>2</v>
+      </c>
+      <c r="E592">
+        <v>8</v>
+      </c>
+      <c r="F592">
+        <v>25</v>
+      </c>
+      <c r="G592" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="593" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A593" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B593" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C593" t="s">
+        <v>103</v>
+      </c>
+      <c r="D593">
+        <v>2</v>
+      </c>
+      <c r="E593">
+        <v>6</v>
+      </c>
+      <c r="F593">
+        <v>30</v>
+      </c>
+      <c r="G593" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="594" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A594" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B594" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C594" t="s">
+        <v>103</v>
+      </c>
+      <c r="D594">
+        <v>3</v>
+      </c>
+      <c r="E594">
+        <v>15</v>
+      </c>
+      <c r="F594">
+        <v>0</v>
+      </c>
+      <c r="G594" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="595" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A595" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B595" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C595" t="s">
+        <v>98</v>
+      </c>
+      <c r="D595">
+        <v>4</v>
+      </c>
+      <c r="E595">
+        <v>8</v>
+      </c>
+      <c r="F595">
+        <v>0</v>
+      </c>
+      <c r="G595" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="596" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A596" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B596" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C596" t="s">
+        <v>105</v>
+      </c>
+      <c r="D596">
+        <v>1</v>
+      </c>
+      <c r="E596">
+        <v>12</v>
+      </c>
+      <c r="F596">
+        <v>0</v>
+      </c>
+      <c r="G596" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="597" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A597" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B597" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C597" t="s">
+        <v>105</v>
+      </c>
+      <c r="D597">
+        <v>1</v>
+      </c>
+      <c r="E597">
+        <v>12</v>
+      </c>
+      <c r="F597">
+        <v>0</v>
+      </c>
+      <c r="G597" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="598" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A598" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B598" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C598" t="s">
+        <v>105</v>
+      </c>
+      <c r="D598">
+        <v>1</v>
+      </c>
+      <c r="E598">
+        <v>12</v>
+      </c>
+      <c r="F598">
+        <v>0</v>
+      </c>
+      <c r="G598" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="599" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A599" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B599" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C599" t="s">
+        <v>103</v>
+      </c>
+      <c r="D599">
+        <v>4</v>
+      </c>
+      <c r="E599">
+        <v>10</v>
+      </c>
+      <c r="F599">
+        <v>20</v>
+      </c>
+      <c r="G599" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="600" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A600" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B600" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C600" t="s">
+        <v>103</v>
+      </c>
+      <c r="D600">
+        <v>5</v>
+      </c>
+      <c r="E600">
+        <v>6</v>
+      </c>
+      <c r="F600">
+        <v>40</v>
+      </c>
+      <c r="G600" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="601" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A601" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B601" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C601" t="s">
+        <v>103</v>
+      </c>
+      <c r="D601">
+        <v>3</v>
+      </c>
+      <c r="E601">
+        <v>15</v>
+      </c>
+      <c r="F601">
+        <v>0</v>
+      </c>
+      <c r="G601" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="602" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A602" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B602" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C602" t="s">
+        <v>103</v>
+      </c>
+      <c r="D602">
+        <v>4</v>
+      </c>
+      <c r="E602">
+        <v>5</v>
+      </c>
+      <c r="F602">
+        <v>0</v>
+      </c>
+      <c r="G602" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="603" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A603" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B603" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C603" t="s">
+        <v>103</v>
+      </c>
+      <c r="D603">
+        <v>3</v>
+      </c>
+      <c r="E603">
+        <v>10</v>
+      </c>
+      <c r="F603">
+        <v>0</v>
+      </c>
+      <c r="G603" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="604" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A604" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B604" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C604" t="s">
+        <v>105</v>
+      </c>
+      <c r="D604">
+        <v>2</v>
+      </c>
+      <c r="E604">
+        <v>15</v>
+      </c>
+      <c r="F604">
+        <v>0</v>
+      </c>
+      <c r="G604" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="605" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A605" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B605" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C605" t="s">
+        <v>105</v>
+      </c>
+      <c r="D605">
+        <v>2</v>
+      </c>
+      <c r="E605">
+        <v>15</v>
+      </c>
+      <c r="F605">
+        <v>0</v>
+      </c>
+      <c r="G605" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="606" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A606" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B606" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C606" t="s">
+        <v>105</v>
+      </c>
+      <c r="D606">
+        <v>1</v>
+      </c>
+      <c r="E606">
+        <v>10</v>
+      </c>
+      <c r="F606">
+        <v>0</v>
+      </c>
+      <c r="G606" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="607" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A607" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B607" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C607" t="s">
+        <v>105</v>
+      </c>
+      <c r="D607">
+        <v>1</v>
+      </c>
+      <c r="E607">
+        <v>15</v>
+      </c>
+      <c r="F607">
+        <v>5</v>
+      </c>
+      <c r="G607" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="608" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A608" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B608" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C608" t="s">
+        <v>104</v>
+      </c>
+      <c r="D608">
+        <v>4</v>
+      </c>
+      <c r="E608">
+        <v>16</v>
+      </c>
+      <c r="F608">
+        <v>0</v>
+      </c>
+      <c r="G608" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="609" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A609" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B609" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C609" t="s">
+        <v>103</v>
+      </c>
+      <c r="D609">
+        <v>1</v>
+      </c>
+      <c r="E609">
+        <v>15</v>
+      </c>
+      <c r="F609">
+        <v>15</v>
+      </c>
+      <c r="G609" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="610" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A610" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B610" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C610" t="s">
+        <v>103</v>
+      </c>
+      <c r="D610">
+        <v>1</v>
+      </c>
+      <c r="E610">
+        <v>15</v>
+      </c>
+      <c r="F610">
+        <v>15</v>
+      </c>
+      <c r="G610" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="611" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A611" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B611" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C611" t="s">
+        <v>103</v>
+      </c>
+      <c r="D611">
+        <v>1</v>
+      </c>
+      <c r="E611">
+        <v>15</v>
+      </c>
+      <c r="F611">
+        <v>15</v>
+      </c>
+      <c r="G611" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="612" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A612" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B612" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C612" t="s">
+        <v>104</v>
+      </c>
+      <c r="D612">
+        <v>4</v>
+      </c>
+      <c r="E612">
+        <v>10</v>
+      </c>
+      <c r="F612">
+        <v>0</v>
+      </c>
+      <c r="G612" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="613" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A613" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B613" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C613" t="s">
+        <v>98</v>
+      </c>
+      <c r="D613">
+        <v>3</v>
+      </c>
+      <c r="E613">
+        <v>25</v>
+      </c>
+      <c r="F613">
+        <v>0</v>
+      </c>
+      <c r="G613" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="614" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A614" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B614" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C614" t="s">
+        <v>103</v>
+      </c>
+      <c r="D614">
+        <v>4</v>
+      </c>
+      <c r="E614">
+        <v>8</v>
+      </c>
+      <c r="F614">
+        <v>70</v>
+      </c>
+      <c r="G614" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="615" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A615" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B615" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C615" t="s">
+        <v>103</v>
+      </c>
+      <c r="D615">
+        <v>4</v>
+      </c>
+      <c r="E615">
+        <v>10</v>
+      </c>
+      <c r="F615">
+        <v>0</v>
+      </c>
+      <c r="G615" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="616" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A616" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B616" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C616" t="s">
+        <v>103</v>
+      </c>
+      <c r="D616">
+        <v>3</v>
+      </c>
+      <c r="E616">
+        <v>6</v>
+      </c>
+      <c r="F616">
+        <v>30</v>
+      </c>
+      <c r="G616" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="617" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A617" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B617" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C617" t="s">
+        <v>105</v>
+      </c>
+      <c r="D617">
+        <v>1</v>
+      </c>
+      <c r="E617">
+        <v>10</v>
+      </c>
+      <c r="F617">
+        <v>0</v>
+      </c>
+      <c r="G617" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="618" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A618" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C618" t="s">
+        <v>105</v>
+      </c>
+      <c r="D618">
+        <v>1</v>
+      </c>
+      <c r="E618">
+        <v>10</v>
+      </c>
+      <c r="F618">
+        <v>0</v>
+      </c>
+      <c r="G618" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="619" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A619" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C619" t="s">
+        <v>103</v>
+      </c>
+      <c r="D619">
+        <v>4</v>
+      </c>
+      <c r="E619">
+        <v>8</v>
+      </c>
+      <c r="F619">
+        <v>110</v>
+      </c>
+      <c r="G619" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="620" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A620" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C620" t="s">
+        <v>103</v>
+      </c>
+      <c r="D620">
+        <v>4</v>
+      </c>
+      <c r="E620">
+        <v>10</v>
+      </c>
+      <c r="F620">
+        <v>115</v>
+      </c>
+      <c r="G620" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="621" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A621" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C621" t="s">
+        <v>103</v>
+      </c>
+      <c r="D621">
+        <v>3</v>
+      </c>
+      <c r="E621">
+        <v>10</v>
+      </c>
+      <c r="F621">
+        <v>25</v>
+      </c>
+      <c r="G621" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="622" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A622" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C622" t="s">
+        <v>103</v>
+      </c>
+      <c r="D622">
+        <v>2</v>
+      </c>
+      <c r="E622">
+        <v>10</v>
+      </c>
+      <c r="F622">
+        <v>230</v>
+      </c>
+      <c r="G622" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="623" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A623" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C623" t="s">
+        <v>103</v>
+      </c>
+      <c r="D623">
+        <v>2</v>
+      </c>
+      <c r="E623">
+        <v>8</v>
+      </c>
+      <c r="F623">
+        <v>270</v>
+      </c>
+      <c r="G623" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="624" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A624" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C624" t="s">
+        <v>103</v>
+      </c>
+      <c r="D624">
+        <v>2</v>
+      </c>
+      <c r="E624">
+        <v>10</v>
+      </c>
+      <c r="F624">
+        <v>15</v>
+      </c>
+      <c r="G624" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A625" s="1">
+        <v>46046</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C625" t="s">
+        <v>103</v>
+      </c>
+      <c r="D625">
+        <v>2</v>
+      </c>
+      <c r="E625">
+        <v>10</v>
+      </c>
+      <c r="F625">
+        <v>25</v>
+      </c>
+      <c r="G625" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="626" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A626" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C626" t="s">
+        <v>98</v>
+      </c>
+      <c r="D626">
+        <v>4</v>
+      </c>
+      <c r="E626">
+        <v>15</v>
+      </c>
+      <c r="F626">
+        <v>0</v>
+      </c>
+      <c r="G626" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="627" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A627" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C627" t="s">
+        <v>104</v>
+      </c>
+      <c r="D627">
+        <v>4</v>
+      </c>
+      <c r="E627">
+        <v>15</v>
+      </c>
+      <c r="F627">
+        <v>0</v>
+      </c>
+      <c r="G627" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="628" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A628" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C628" t="s">
+        <v>104</v>
+      </c>
+      <c r="D628">
+        <v>4</v>
+      </c>
+      <c r="E628">
+        <v>15</v>
+      </c>
+      <c r="F628">
+        <v>0</v>
+      </c>
+      <c r="G628" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="629" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A629" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C629" t="s">
+        <v>104</v>
+      </c>
+      <c r="D629">
+        <v>3</v>
+      </c>
+      <c r="E629">
+        <v>25</v>
+      </c>
+      <c r="F629">
+        <v>0</v>
+      </c>
+      <c r="G629" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="630" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A630" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C630" t="s">
+        <v>98</v>
+      </c>
+      <c r="D630">
+        <v>4</v>
+      </c>
+      <c r="E630">
+        <v>10</v>
+      </c>
+      <c r="F630">
+        <v>0</v>
+      </c>
+      <c r="G630" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="631" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A631" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="C631" t="s">
+        <v>103</v>
+      </c>
+      <c r="D631">
+        <v>5</v>
+      </c>
+      <c r="E631">
+        <v>5</v>
+      </c>
+      <c r="F631">
+        <v>30</v>
+      </c>
+      <c r="G631" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="632" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A632" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C632" t="s">
+        <v>103</v>
+      </c>
+      <c r="D632">
+        <v>3</v>
+      </c>
+      <c r="E632">
+        <v>5</v>
+      </c>
+      <c r="F632">
+        <v>0</v>
+      </c>
+      <c r="G632" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="633" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A633" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B633" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C633" t="s">
+        <v>105</v>
+      </c>
+      <c r="D633">
+        <v>2</v>
+      </c>
+      <c r="E633">
+        <v>15</v>
+      </c>
+      <c r="F633">
+        <v>0</v>
+      </c>
+      <c r="G633" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="634" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A634" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B634" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C634" t="s">
+        <v>105</v>
+      </c>
+      <c r="D634">
+        <v>2</v>
+      </c>
+      <c r="E634">
+        <v>15</v>
+      </c>
+      <c r="F634">
+        <v>0</v>
+      </c>
+      <c r="G634" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="635" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A635" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B635" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C635" t="s">
+        <v>105</v>
+      </c>
+      <c r="D635">
+        <v>1</v>
+      </c>
+      <c r="E635">
+        <v>10</v>
+      </c>
+      <c r="F635">
+        <v>0</v>
+      </c>
+      <c r="G635" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -14750,7 +16191,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C015AB5-FA38-994A-89E4-279E0D11AC16}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -14948,6 +16389,40 @@
       </c>
       <c r="E11">
         <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B12" t="s">
+        <v>188</v>
+      </c>
+      <c r="C12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D12" t="s">
+        <v>187</v>
+      </c>
+      <c r="E12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>46049</v>
+      </c>
+      <c r="B13" t="s">
+        <v>207</v>
+      </c>
+      <c r="C13" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" t="s">
+        <v>187</v>
+      </c>
+      <c r="E13">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>